<commit_message>
Updated code for upload and prepare dataset for HF
</commit_message>
<xml_diff>
--- a/evaluation_sheet.xlsx
+++ b/evaluation_sheet.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3350,6 +3350,336 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>source_attribution</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>2</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Cites only a generic 'government schemes information' without a concrete, verifiable source or link. While the claim aligns with the retrieved scheme list, the response does not explicitly attribute to that list or any official document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>grammatical_accuracy</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>3</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Mostly clear Marathi, but contains noticeable lexical/usage issues such as 'शेतभाताच्या कुंपणासाठी' (incorrect; should be 'शेताभोवतीच्या कुंपणासाठी') and minor register inconsistencies (e.g., 'निकटच्या').</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>factual_correctness</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>4</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Consistent with the retrieved list that does not show a dedicated 'Solar Fencing Scheme' for Maharashtra. No apparent false claims, though the statement is broad and could overlook district/departmental programs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>actionability</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Provides only generic advice to contact local offices; lacks concrete steps, portals (e.g., state application portals), eligibility, documents, timelines, or process details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>completeness</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>2</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Acknowledges the query and notes non-availability but does not cover possible related schemes, alternative support channels, or detailed guidance. No follow-up questions to refine assistance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>context_alignment</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Addresses the user’s intent about a solar fencing scheme, but response is generic and does not deeply engage with the specific needs implied by the query.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>information</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Information is minimal and generic. Lacks specifics on subsidies, application procedures, or verification steps (e.g., checking official portals), reducing practical value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>safety_compliance</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>5</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>No unsafe or non-compliant practices recommended. Advice to consult official authorities is safe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>tool_usage</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>4</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Used a relevant tool to retrieve scheme listings and based the response on it. Could have better leveraged the tool output by explicitly referencing items or guiding next steps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>सौर कुंपण योजना</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>आपण विचारलेली "सौर कुंपण योजना" (Solar Fencing Scheme) नावाची कृषी योजना सद्यस्थितीत महाराष्ट्रातील अधिकृत शासकीय योजना यादीमध्ये स्वतंत्रपणे उपलब्ध नाही. सध्या शेतकऱ्यांसाठी देण्यात येणाऱ्या महत्त्वाच्या राज्य व केंद्र सरकारच्या योजना वरील यादीत दिल्या आहेत. त्यामध्ये सिंचन, शेती यंत्रसामुग्री, पाणी व्यवस्थापन, सुरक्षा, व इतर विविध शेती सुधारणा संबंधित योजना आहेत.
+जर आपल्याला शेतभाताच्या कुंपणासाठी (फेन्सिंग) किंवा सौरऊर्जेवर चालणाऱ्या कुंपणासाठी शासकीय अनुदानाची माहिती हवी असेल, तर कृपया आपले जिल्हा किंवा तालुका कृषी कार्यालय, ग्रामपंचायत, किंवा निकटच्या कृषी विज्ञान केंद्रात संपर्क साधा. काही वेळा राज्य किंवा केंद्र सरकारकडून विशेष निधी, समिती, किंवा जिल्हास्तरावर प्रायोगिक योजना जाहीर केल्या जातात, त्या बद्दल स्थानिक कृषी अधिकार्‍यांशी विचारणा करा.
+आपल्याला अन्य कोणती शासकीय योजना किंवा अनुदानाची माहिती हवी असेल का? मी महाराष्ट्रातील उपलब्ध कृषी योजनांची अधिकृत माहिती सुद्धा देऊ शकतो.
+**स्रोत: शासकीय योजना माहिती**</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Marathi</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>retrieval_grounding</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>4</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Predominantly grounded in the retrieved scheme list; avoids speculation. However, the broad non-availability claim could benefit from explicit linkage to the retrieved data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>